<commit_message>
Preserve experiment code and finalize submission presentation
</commit_message>
<xml_diff>
--- a/submissions/2A202602800_NguyenVanHong/results.xlsx
+++ b/submissions/2A202602800_NguyenVanHong/results.xlsx
@@ -16,7 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backbones'!$A$1:$U$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backbones'!$A$1:$V$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Training'!$A$1:$AA$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Inference'!$A$1:$N$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Final'!$A$1:$I$11</definedName>
@@ -89,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -117,6 +117,12 @@
     </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -483,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:V6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -507,6 +513,7 @@
     <col width="15" customWidth="1" min="19" max="19"/>
     <col width="23" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="42" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -615,6 +622,11 @@
           <t>gpu</t>
         </is>
       </c>
+      <c r="V1" s="12" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -692,6 +704,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="V2" s="13" t="inlineStr">
+        <is>
+          <t>Common recipe, 12 epochs, seed 0; preliminary FP32 batch-1 latency</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -769,6 +786,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="V3" s="13" t="inlineStr">
+        <is>
+          <t>Common recipe, 12 epochs, seed 0; preliminary FP32 batch-1 latency</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -846,6 +868,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="V4" s="13" t="inlineStr">
+        <is>
+          <t>Common recipe, 12 epochs, seed 0; preliminary FP32 batch-1 latency</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -923,6 +950,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="V5" s="13" t="inlineStr">
+        <is>
+          <t>Common recipe, 12 epochs, seed 0; preliminary FP32 batch-1 latency</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1000,9 +1032,14 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="V6" s="13" t="inlineStr">
+        <is>
+          <t>Common recipe, 12 epochs, seed 0; preliminary FP32 batch-1 latency</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U6"/>
+  <autoFilter ref="A1:V6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>